<commit_message>
MultiSport: add per-team effort dial (0-100) scaling spend across worst/contender/national anchors
Each team row has a 0-100 dial; 0=worst-in-conf, 50=conference contender (= prior base),
100=national contender. Benchmark engine interpolates op cost, team revenue, and athlete
comp (split rev-share/NIL) per dial. FCS/FBS football toggle retained. All-@50 reproduces
$23.5M all-in / -$18.2M net.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ajJRqKa1DUy4iKHJKPEi3
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-30-cinderella-model-d3-multisport.xlsx
+++ b/cinderella/Outputs/2026-07-30-cinderella-model-d3-multisport.xlsx
@@ -91,7 +91,7 @@
     <numFmt numFmtId="168" formatCode="$#,##0;($#,##0);-"/>
     <numFmt numFmtId="169" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -292,8 +292,9 @@
       <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
+    <font/>
   </fonts>
-  <fills count="18">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -388,6 +389,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
   </fills>
@@ -638,7 +649,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="217">
+  <cellXfs count="229">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1202,6 +1213,26 @@
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="35" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="35" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="33" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="34" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="34" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="35" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="35" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -46766,12 +46797,12 @@
           <t>Equity holder (share of 6-yr net CF)</t>
         </is>
       </c>
-      <c r="C60" s="205" t="inlineStr">
+      <c r="C60" s="216" t="inlineStr">
         <is>
           <t>Equity %</t>
         </is>
       </c>
-      <c r="I60" s="205" t="inlineStr">
+      <c r="I60" s="216" t="inlineStr">
         <is>
           <t>6-yr $ to holder</t>
         </is>
@@ -46961,690 +46992,952 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:K46"/>
+  <dimension ref="B1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="174" min="1" max="1"/>
-    <col width="24" customWidth="1" style="174" min="2" max="2"/>
-    <col width="15" customWidth="1" style="174" min="3" max="3"/>
-    <col width="15" customWidth="1" style="174" min="4" max="4"/>
-    <col width="15" customWidth="1" style="174" min="5" max="5"/>
-    <col width="15" customWidth="1" style="174" min="6" max="6"/>
-    <col width="15" customWidth="1" style="174" min="7" max="7"/>
-    <col width="15" customWidth="1" style="174" min="8" max="8"/>
-    <col width="15" customWidth="1" style="174" min="9" max="9"/>
-    <col width="50" customWidth="1" style="174" min="11" max="11"/>
+    <col width="22" customWidth="1" style="174" min="2" max="2"/>
+    <col width="11" customWidth="1" style="174" min="3" max="3"/>
+    <col width="14" customWidth="1" style="174" min="4" max="4"/>
+    <col width="14" customWidth="1" style="174" min="5" max="5"/>
+    <col width="14" customWidth="1" style="174" min="6" max="6"/>
+    <col width="14" customWidth="1" style="174" min="7" max="7"/>
+    <col width="14" customWidth="1" style="174" min="8" max="8"/>
+    <col width="14" customWidth="1" style="174" min="9" max="9"/>
+    <col width="14" customWidth="1" style="174" min="10" max="10"/>
+    <col width="46" customWidth="1" style="174" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="B1" s="185" t="inlineStr">
         <is>
-          <t>MULTI-SPORT PROGRAM — D1 CONFERENCE-COMPETITIVE ECONOMICS</t>
+          <t>MULTI-SPORT PROGRAM — EFFORT-DIALED D1 ECONOMICS</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="186" t="inlineStr">
         <is>
-          <t>Per-sport annual steady-state to be BEST IN A LOW/MID-MAJOR D1 CONFERENCE (not national-title). Post-House era: athlete pay = revenue-share (school) + NIL (third party).</t>
+          <t>Per-team EFFORT dial (0-100) scales spend:  0 = worst in a bottom-tier D1 league  ·  50 = conference-title contender  ·  100 = national-championship contender.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="186" t="inlineStr">
         <is>
-          <t>Blue = editable input. The four shaded columns (C–F) are the story Norman asked for. Team revenue here is BASE athletics only — Making Cinderella content/sponsor upside is in the SPV tabs and layers on top.</t>
+          <t>Set each team's dial (orange). The four story columns (blue) compute from it. Team revenue = base athletics only; Making Cinderella content/sponsor upside is in the SPV tabs and layers on top.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="197" t="inlineStr">
+      <c r="B5" s="187" t="inlineStr">
         <is>
-          <t>Football level (type FCS or FBS):</t>
+          <t>SCALING &amp; GLOBAL INPUTS  (blue = editable)</t>
         </is>
       </c>
-      <c r="C5" s="209" t="inlineStr">
+      <c r="C5" s="199" t="inlineStr"/>
+      <c r="D5" s="199" t="inlineStr"/>
+      <c r="E5" s="199" t="inlineStr"/>
+      <c r="F5" s="199" t="inlineStr"/>
+      <c r="G5" s="199" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="193" t="inlineStr">
+        <is>
+          <t>Op-cost scale — factor @0 / @100 effort</t>
+        </is>
+      </c>
+      <c r="C6" s="217" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D6" s="217" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="L6" s="192" t="inlineStr">
+        <is>
+          <t>Op cost has a high floor (you still pay coaches/travel/scholars) and rises to elite staff+facilities at 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="193" t="inlineStr">
+        <is>
+          <t>Team-revenue scale — factor @0 / @100</t>
+        </is>
+      </c>
+      <c r="C7" s="217" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D7" s="217" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L7" s="192" t="inlineStr">
+        <is>
+          <t>Winning earns more (tickets, guarantees, units). Big content/unit upside is captured in the SPV tabs, not here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="193" t="inlineStr">
+        <is>
+          <t>House rev-share cap (2025-26 ref)</t>
+        </is>
+      </c>
+      <c r="C8" s="207" t="n">
+        <v>20500000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="193" t="inlineStr">
+        <is>
+          <t>Football level (type FCS or FBS)</t>
+        </is>
+      </c>
+      <c r="C9" s="218" t="inlineStr">
         <is>
           <t>FCS</t>
         </is>
       </c>
-      <c r="K5" s="192" t="inlineStr">
+      <c r="L9" s="192" t="inlineStr">
         <is>
-          <t>FCS = realistic reclassification path. FBS = far costlier + harder to qualify; drives the Football row from the scenario block (rows 34-37).</t>
+          <t>FCS = realistic reclassification path. FBS = far costlier/harder; drives the Football engine row.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="197" t="inlineStr">
+    <row r="11" ht="30" customHeight="1" s="174">
+      <c r="B11" s="187" t="inlineStr">
         <is>
-          <t>House revenue-share cap (2025-26 ref):</t>
+          <t>TEAM</t>
         </is>
       </c>
-      <c r="C6" s="207" t="n">
-        <v>20500000</v>
-      </c>
-      <c r="K6" s="192" t="inlineStr">
+      <c r="C11" s="210" t="inlineStr">
         <is>
-          <t>Per-school cap on DIRECT school-&gt;athlete pay (rev-share). NIL sits on top. Rises ~4%/yr.</t>
+          <t>EFFORT
+0-100</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="30" customHeight="1" s="174">
-      <c r="B8" s="187" t="inlineStr">
-        <is>
-          <t>SPORT</t>
-        </is>
-      </c>
-      <c r="C8" s="210" t="inlineStr">
+      <c r="D11" s="210" t="inlineStr">
         <is>
           <t>1 · Total op. costs</t>
         </is>
       </c>
-      <c r="D8" s="210" t="inlineStr">
+      <c r="E11" s="210" t="inlineStr">
         <is>
           <t>2 · Total team revenue</t>
         </is>
       </c>
-      <c r="E8" s="210" t="inlineStr">
+      <c r="F11" s="210" t="inlineStr">
         <is>
-          <t>3 · Athlete rev-share (comp)</t>
+          <t>3 · Athlete rev-share</t>
         </is>
       </c>
-      <c r="F8" s="210" t="inlineStr">
+      <c r="G11" s="210" t="inlineStr">
         <is>
-          <t>4 · NIL 3rd-party (comp)</t>
+          <t>4 · NIL 3rd-party</t>
         </is>
       </c>
-      <c r="G8" s="210" t="inlineStr">
+      <c r="H11" s="210" t="inlineStr">
         <is>
           <t>Athlete comp (3+4)</t>
         </is>
       </c>
-      <c r="H8" s="210" t="inlineStr">
+      <c r="I11" s="210" t="inlineStr">
         <is>
           <t>All-in cost (1+3+4)</t>
         </is>
       </c>
-      <c r="I8" s="210" t="inlineStr">
+      <c r="J11" s="210" t="inlineStr">
         <is>
           <t>Net (2 − all-in)</t>
         </is>
       </c>
-      <c r="K8" s="187" t="inlineStr">
+      <c r="L11" s="187" t="inlineStr">
         <is>
           <t>BASIS / SOURCE</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="197" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="197" t="inlineStr">
         <is>
           <t>Football</t>
         </is>
       </c>
-      <c r="C9" s="211">
-        <f>IF($C$5="FBS",C37,C36)</f>
-        <v/>
-      </c>
-      <c r="D9" s="211">
-        <f>IF($C$5="FBS",D37,D36)</f>
-        <v/>
-      </c>
-      <c r="E9" s="211">
-        <f>IF($C$5="FBS",E37,E36)</f>
-        <v/>
-      </c>
-      <c r="F9" s="211">
-        <f>IF($C$5="FBS",F37,F36)</f>
-        <v/>
-      </c>
-      <c r="G9" s="212">
-        <f>E9+F9</f>
-        <v/>
-      </c>
-      <c r="H9" s="212">
-        <f>C9+E9+F9</f>
-        <v/>
-      </c>
-      <c r="I9" s="212">
-        <f>D9-H9</f>
-        <v/>
-      </c>
-      <c r="K9" s="192" t="inlineStr">
+      <c r="C12" s="219" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" s="211">
+        <f>C26*IF(C12&lt;=50,$C$6+(1-$C$6)*C12/50,1+($D$6-1)*(C12-50)/50)</f>
+        <v/>
+      </c>
+      <c r="E12" s="211">
+        <f>D26*IF(C12&lt;=50,$C$7+(1-$C$7)*C12/50,1+($D$7-1)*(C12-50)/50)</f>
+        <v/>
+      </c>
+      <c r="F12" s="211">
+        <f>H12*H26</f>
+        <v/>
+      </c>
+      <c r="G12" s="211">
+        <f>H12-F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="212">
+        <f>IF(C12&lt;=50,E26+(F26-E26)*C12/50,F26+(G26-F26)*(C12-50)/50)</f>
+        <v/>
+      </c>
+      <c r="I12" s="212">
+        <f>D12+H12</f>
+        <v/>
+      </c>
+      <c r="J12" s="212">
+        <f>E12-I12</f>
+        <v/>
+      </c>
+      <c r="L12" s="192" t="inlineStr">
         <is>
-          <t>FCS toggled from scenario block. FCS NIL still nascent; top FCS op-budgets ~$9-13M. $20M+ = FBS.</t>
+          <t>FCS toggled. FCS NIL nascent; top FCS op-budgets ~$9-13M. $20M+ implies FBS.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="197" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="197" t="inlineStr">
         <is>
           <t>Men's Basketball</t>
         </is>
       </c>
-      <c r="C10" s="213" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="D10" s="213" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="E10" s="213" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="F10" s="213" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="G10" s="212">
-        <f>E10+F10</f>
-        <v/>
-      </c>
-      <c r="H10" s="212">
-        <f>C10+E10+F10</f>
-        <v/>
-      </c>
-      <c r="I10" s="212">
-        <f>D10-H10</f>
-        <v/>
-      </c>
-      <c r="K10" s="192" t="inlineStr">
+      <c r="C13" s="219" t="n">
+        <v>50</v>
+      </c>
+      <c r="D13" s="211">
+        <f>C27*IF(C13&lt;=50,$C$6+(1-$C$6)*C13/50,1+($D$6-1)*(C13-50)/50)</f>
+        <v/>
+      </c>
+      <c r="E13" s="211">
+        <f>D27*IF(C13&lt;=50,$C$7+(1-$C$7)*C13/50,1+($D$7-1)*(C13-50)/50)</f>
+        <v/>
+      </c>
+      <c r="F13" s="211">
+        <f>H13*H27</f>
+        <v/>
+      </c>
+      <c r="G13" s="211">
+        <f>H13-F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="212">
+        <f>IF(C13&lt;=50,E27+(F27-E27)*C13/50,F27+(G27-F27)*(C13-50)/50)</f>
+        <v/>
+      </c>
+      <c r="I13" s="212">
+        <f>D13+H13</f>
+        <v/>
+      </c>
+      <c r="J13" s="212">
+        <f>E13-I13</f>
+        <v/>
+      </c>
+      <c r="L13" s="192" t="inlineStr">
         <is>
-          <t>Mid-major 'C-tier' rosters $1-2M; $2.5M tops a one-bid league. The Cinderella flagship.</t>
+          <t>The Cinderella flagship. @50 tops a one-bid league; @100 = ~$12M top-25 (matches SPV).</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="197" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="197" t="inlineStr">
         <is>
           <t>Women's Basketball</t>
         </is>
       </c>
-      <c r="C11" s="213" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="D11" s="213" t="n">
-        <v>400000</v>
-      </c>
-      <c r="E11" s="213" t="n">
-        <v>600000</v>
-      </c>
-      <c r="F11" s="213" t="n">
-        <v>400000</v>
-      </c>
-      <c r="G11" s="212">
-        <f>E11+F11</f>
-        <v/>
-      </c>
-      <c r="H11" s="212">
-        <f>C11+E11+F11</f>
-        <v/>
-      </c>
-      <c r="I11" s="212">
-        <f>D11-H11</f>
-        <v/>
-      </c>
-      <c r="K11" s="192" t="inlineStr">
+      <c r="C14" s="219" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" s="211">
+        <f>C28*IF(C14&lt;=50,$C$6+(1-$C$6)*C14/50,1+($D$6-1)*(C14-50)/50)</f>
+        <v/>
+      </c>
+      <c r="E14" s="211">
+        <f>D28*IF(C14&lt;=50,$C$7+(1-$C$7)*C14/50,1+($D$7-1)*(C14-50)/50)</f>
+        <v/>
+      </c>
+      <c r="F14" s="211">
+        <f>H14*H28</f>
+        <v/>
+      </c>
+      <c r="G14" s="211">
+        <f>H14-F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="212">
+        <f>IF(C14&lt;=50,E28+(F28-E28)*C14/50,F28+(G28-F28)*(C14-50)/50)</f>
+        <v/>
+      </c>
+      <c r="I14" s="212">
+        <f>D14+H14</f>
+        <v/>
+      </c>
+      <c r="J14" s="212">
+        <f>E14-I14</f>
+        <v/>
+      </c>
+      <c r="L14" s="192" t="inlineStr">
         <is>
-          <t>American 'war chest' $0.75-1.5M; Sun Belt entry $250-500K. Rev-share avg ~$1.4M at opt-in schools.</t>
+          <t>@50 ~ American 'war chest'; rev-share avg ~$1.4M at opt-in schools.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="197" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="197" t="inlineStr">
         <is>
           <t>Baseball</t>
         </is>
       </c>
-      <c r="C12" s="213" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="D12" s="213" t="n">
-        <v>400000</v>
-      </c>
-      <c r="E12" s="213" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F12" s="213" t="n">
-        <v>350000</v>
-      </c>
-      <c r="G12" s="212">
-        <f>E12+F12</f>
-        <v/>
-      </c>
-      <c r="H12" s="212">
-        <f>C12+E12+F12</f>
-        <v/>
-      </c>
-      <c r="I12" s="212">
-        <f>D12-H12</f>
-        <v/>
-      </c>
-      <c r="K12" s="192" t="inlineStr">
+      <c r="C15" s="219" t="n">
+        <v>50</v>
+      </c>
+      <c r="D15" s="211">
+        <f>C29*IF(C15&lt;=50,$C$6+(1-$C$6)*C15/50,1+($D$6-1)*(C15-50)/50)</f>
+        <v/>
+      </c>
+      <c r="E15" s="211">
+        <f>D29*IF(C15&lt;=50,$C$7+(1-$C$7)*C15/50,1+($D$7-1)*(C15-50)/50)</f>
+        <v/>
+      </c>
+      <c r="F15" s="211">
+        <f>H15*H29</f>
+        <v/>
+      </c>
+      <c r="G15" s="211">
+        <f>H15-F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="212">
+        <f>IF(C15&lt;=50,E29+(F29-E29)*C15/50,F29+(G29-F29)*(C15-50)/50)</f>
+        <v/>
+      </c>
+      <c r="I15" s="212">
+        <f>D15+H15</f>
+        <v/>
+      </c>
+      <c r="J15" s="212">
+        <f>E15-I15</f>
+        <v/>
+      </c>
+      <c r="L15" s="192" t="inlineStr">
         <is>
-          <t>Now up to 34 full scholarships; NIL market thin. Won more by scholarships/facilities.</t>
+          <t>Up to 34 full scholarships now; NIL thin — won via scholarships/facilities.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="197" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="197" t="inlineStr">
         <is>
           <t>Softball</t>
         </is>
       </c>
-      <c r="C13" s="213" t="n">
-        <v>800000</v>
-      </c>
-      <c r="D13" s="213" t="n">
-        <v>200000</v>
-      </c>
-      <c r="E13" s="213" t="n">
-        <v>400000</v>
-      </c>
-      <c r="F13" s="213" t="n">
-        <v>200000</v>
-      </c>
-      <c r="G13" s="212">
-        <f>E13+F13</f>
-        <v/>
-      </c>
-      <c r="H13" s="212">
-        <f>C13+E13+F13</f>
-        <v/>
-      </c>
-      <c r="I13" s="212">
-        <f>D13-H13</f>
-        <v/>
-      </c>
-      <c r="K13" s="192" t="inlineStr">
+      <c r="C16" s="219" t="n">
+        <v>50</v>
+      </c>
+      <c r="D16" s="211">
+        <f>C30*IF(C16&lt;=50,$C$6+(1-$C$6)*C16/50,1+($D$6-1)*(C16-50)/50)</f>
+        <v/>
+      </c>
+      <c r="E16" s="211">
+        <f>D30*IF(C16&lt;=50,$C$7+(1-$C$7)*C16/50,1+($D$7-1)*(C16-50)/50)</f>
+        <v/>
+      </c>
+      <c r="F16" s="211">
+        <f>H16*H30</f>
+        <v/>
+      </c>
+      <c r="G16" s="211">
+        <f>H16-F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="212">
+        <f>IF(C16&lt;=50,E30+(F30-E30)*C16/50,F30+(G30-F30)*(C16-50)/50)</f>
+        <v/>
+      </c>
+      <c r="I16" s="212">
+        <f>D16+H16</f>
+        <v/>
+      </c>
+      <c r="J16" s="212">
+        <f>E16-I16</f>
+        <v/>
+      </c>
+      <c r="L16" s="192" t="inlineStr">
         <is>
           <t>Thin NIL; competitive via scholarships + coaching.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="197" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="197" t="inlineStr">
         <is>
           <t>Men's Soccer</t>
         </is>
       </c>
-      <c r="C14" s="213" t="n">
-        <v>700000</v>
-      </c>
-      <c r="D14" s="213" t="n">
-        <v>150000</v>
-      </c>
-      <c r="E14" s="213" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F14" s="213" t="n">
-        <v>200000</v>
-      </c>
-      <c r="G14" s="212">
-        <f>E14+F14</f>
-        <v/>
-      </c>
-      <c r="H14" s="212">
-        <f>C14+E14+F14</f>
-        <v/>
-      </c>
-      <c r="I14" s="212">
-        <f>D14-H14</f>
-        <v/>
-      </c>
-      <c r="K14" s="192" t="inlineStr">
+      <c r="C17" s="219" t="n">
+        <v>50</v>
+      </c>
+      <c r="D17" s="211">
+        <f>C31*IF(C17&lt;=50,$C$6+(1-$C$6)*C17/50,1+($D$6-1)*(C17-50)/50)</f>
+        <v/>
+      </c>
+      <c r="E17" s="211">
+        <f>D31*IF(C17&lt;=50,$C$7+(1-$C$7)*C17/50,1+($D$7-1)*(C17-50)/50)</f>
+        <v/>
+      </c>
+      <c r="F17" s="211">
+        <f>H17*H31</f>
+        <v/>
+      </c>
+      <c r="G17" s="211">
+        <f>H17-F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="212">
+        <f>IF(C17&lt;=50,E31+(F31-E31)*C17/50,F31+(G31-F31)*(C17-50)/50)</f>
+        <v/>
+      </c>
+      <c r="I17" s="212">
+        <f>D17+H17</f>
+        <v/>
+      </c>
+      <c r="J17" s="212">
+        <f>E17-I17</f>
+        <v/>
+      </c>
+      <c r="L17" s="192" t="inlineStr">
         <is>
           <t>Low-major; modest NIL, diminishing returns.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="197" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="197" t="inlineStr">
         <is>
           <t>Women's Soccer</t>
         </is>
       </c>
-      <c r="C15" s="213" t="n">
-        <v>700000</v>
-      </c>
-      <c r="D15" s="213" t="n">
-        <v>150000</v>
-      </c>
-      <c r="E15" s="213" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F15" s="213" t="n">
-        <v>150000</v>
-      </c>
-      <c r="G15" s="212">
-        <f>E15+F15</f>
-        <v/>
-      </c>
-      <c r="H15" s="212">
-        <f>C15+E15+F15</f>
-        <v/>
-      </c>
-      <c r="I15" s="212">
-        <f>D15-H15</f>
-        <v/>
-      </c>
-      <c r="K15" s="192" t="inlineStr">
+      <c r="C18" s="219" t="n">
+        <v>50</v>
+      </c>
+      <c r="D18" s="211">
+        <f>C32*IF(C18&lt;=50,$C$6+(1-$C$6)*C18/50,1+($D$6-1)*(C18-50)/50)</f>
+        <v/>
+      </c>
+      <c r="E18" s="211">
+        <f>D32*IF(C18&lt;=50,$C$7+(1-$C$7)*C18/50,1+($D$7-1)*(C18-50)/50)</f>
+        <v/>
+      </c>
+      <c r="F18" s="211">
+        <f>H18*H32</f>
+        <v/>
+      </c>
+      <c r="G18" s="211">
+        <f>H18-F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="212">
+        <f>IF(C18&lt;=50,E32+(F32-E32)*C18/50,F32+(G32-F32)*(C18-50)/50)</f>
+        <v/>
+      </c>
+      <c r="I18" s="212">
+        <f>D18+H18</f>
+        <v/>
+      </c>
+      <c r="J18" s="212">
+        <f>E18-I18</f>
+        <v/>
+      </c>
+      <c r="L18" s="192" t="inlineStr">
         <is>
           <t>Low-major; modest NIL.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="197" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="197" t="inlineStr">
         <is>
           <t>Men's Lacrosse</t>
         </is>
       </c>
-      <c r="C16" s="213" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="D16" s="213" t="n">
-        <v>300000</v>
-      </c>
-      <c r="E16" s="213" t="n">
-        <v>350000</v>
-      </c>
-      <c r="F16" s="213" t="n">
-        <v>250000</v>
-      </c>
-      <c r="G16" s="212">
-        <f>E16+F16</f>
-        <v/>
-      </c>
-      <c r="H16" s="212">
-        <f>C16+E16+F16</f>
-        <v/>
-      </c>
-      <c r="I16" s="212">
-        <f>D16-H16</f>
-        <v/>
-      </c>
-      <c r="K16" s="192" t="inlineStr">
+      <c r="C19" s="219" t="n">
+        <v>50</v>
+      </c>
+      <c r="D19" s="211">
+        <f>C33*IF(C19&lt;=50,$C$6+(1-$C$6)*C19/50,1+($D$6-1)*(C19-50)/50)</f>
+        <v/>
+      </c>
+      <c r="E19" s="211">
+        <f>D33*IF(C19&lt;=50,$C$7+(1-$C$7)*C19/50,1+($D$7-1)*(C19-50)/50)</f>
+        <v/>
+      </c>
+      <c r="F19" s="211">
+        <f>H19*H33</f>
+        <v/>
+      </c>
+      <c r="G19" s="211">
+        <f>H19-F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="212">
+        <f>IF(C19&lt;=50,E33+(F33-E33)*C19/50,F33+(G33-F33)*(C19-50)/50)</f>
+        <v/>
+      </c>
+      <c r="I19" s="212">
+        <f>D19+H19</f>
+        <v/>
+      </c>
+      <c r="J19" s="212">
+        <f>E19-I19</f>
+        <v/>
+      </c>
+      <c r="L19" s="192" t="inlineStr">
         <is>
-          <t>Regional recruiting (a JHU-tier build); niche NIL market.</t>
+          <t>Regional (JHU-tier build); niche NIL market.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="197" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="197" t="inlineStr">
         <is>
           <t>Women's Lacrosse</t>
         </is>
       </c>
-      <c r="C17" s="213" t="n">
-        <v>800000</v>
-      </c>
-      <c r="D17" s="213" t="n">
-        <v>200000</v>
-      </c>
-      <c r="E17" s="213" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F17" s="213" t="n">
-        <v>150000</v>
-      </c>
-      <c r="G17" s="212">
-        <f>E17+F17</f>
-        <v/>
-      </c>
-      <c r="H17" s="212">
-        <f>C17+E17+F17</f>
-        <v/>
-      </c>
-      <c r="I17" s="212">
-        <f>D17-H17</f>
-        <v/>
-      </c>
-      <c r="K17" s="192" t="inlineStr">
+      <c r="C20" s="219" t="n">
+        <v>50</v>
+      </c>
+      <c r="D20" s="211">
+        <f>C34*IF(C20&lt;=50,$C$6+(1-$C$6)*C20/50,1+($D$6-1)*(C20-50)/50)</f>
+        <v/>
+      </c>
+      <c r="E20" s="211">
+        <f>D34*IF(C20&lt;=50,$C$7+(1-$C$7)*C20/50,1+($D$7-1)*(C20-50)/50)</f>
+        <v/>
+      </c>
+      <c r="F20" s="211">
+        <f>H20*H34</f>
+        <v/>
+      </c>
+      <c r="G20" s="211">
+        <f>H20-F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="212">
+        <f>IF(C20&lt;=50,E34+(F34-E34)*C20/50,F34+(G34-F34)*(C20-50)/50)</f>
+        <v/>
+      </c>
+      <c r="I20" s="212">
+        <f>D20+H20</f>
+        <v/>
+      </c>
+      <c r="J20" s="212">
+        <f>E20-I20</f>
+        <v/>
+      </c>
+      <c r="L20" s="192" t="inlineStr">
         <is>
           <t>Regional; niche NIL market.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="203" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="203" t="inlineStr">
         <is>
-          <t>TOTAL (all 9 sports)</t>
+          <t>TOTAL (program)</t>
         </is>
       </c>
-      <c r="C18" s="204">
-        <f>SUM(C9:C17)</f>
-        <v/>
-      </c>
-      <c r="D18" s="204">
-        <f>SUM(D9:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="204">
-        <f>SUM(E9:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="204">
-        <f>SUM(F9:F17)</f>
-        <v/>
-      </c>
-      <c r="G18" s="204">
-        <f>SUM(G9:G17)</f>
-        <v/>
-      </c>
-      <c r="H18" s="204">
-        <f>SUM(H9:H17)</f>
-        <v/>
-      </c>
-      <c r="I18" s="204">
-        <f>SUM(I9:I17)</f>
-        <v/>
-      </c>
-      <c r="K18" s="186" t="inlineStr">
+      <c r="C21" s="220" t="inlineStr"/>
+      <c r="D21" s="204">
+        <f>SUM(D12:D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="204">
+        <f>SUM(E12:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="204">
+        <f>SUM(F12:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="204">
+        <f>SUM(G12:G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="204">
+        <f>SUM(H12:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="204">
+        <f>SUM(I12:I20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="204">
+        <f>SUM(J12:J20)</f>
+        <v/>
+      </c>
+      <c r="L21" s="186" t="inlineStr">
         <is>
-          <t>Steady-state, conference-best across every sport.</t>
+          <t>Sum across all teams at their current dial settings.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="187" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="186" t="inlineStr">
+        <is>
+          <t>Dial guide:  0 = worst in conference   ·   50 = conference-title contender   ·   100 = national-championship contender</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="187" t="inlineStr">
         <is>
           <t>SUMMARY</t>
         </is>
       </c>
-      <c r="C20" s="199" t="inlineStr"/>
-      <c r="D20" s="199" t="inlineStr"/>
-      <c r="E20" s="199" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="193" t="inlineStr">
+      <c r="C24" s="199" t="inlineStr"/>
+      <c r="D24" s="199" t="inlineStr"/>
+    </row>
+    <row r="25" ht="26" customHeight="1" s="174">
+      <c r="B25" s="221" t="inlineStr">
         <is>
-          <t>Total athlete comp (rev-share + NIL)</t>
+          <t>BENCHMARK ENGINE  (blue = editable $ anchors that the dials interpolate)</t>
         </is>
       </c>
-      <c r="C21" s="201">
-        <f>G18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="193" t="inlineStr">
+      <c r="C25" s="222" t="inlineStr">
         <is>
-          <t>Total rev-share vs House cap</t>
+          <t>op base@50</t>
         </is>
       </c>
-      <c r="C22" s="201">
-        <f>E18</f>
-        <v/>
-      </c>
-      <c r="D22" s="193">
-        <f>IF(E18&gt;C6,"OVER CAP — needs waiver/collective","under cap — headroom remains")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="193" t="inlineStr">
+      <c r="D25" s="223" t="inlineStr">
         <is>
-          <t>Total all-in program cost (op + comp)</t>
+          <t>rev base@50</t>
         </is>
       </c>
-      <c r="C23" s="201">
-        <f>H18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="197" t="inlineStr">
+      <c r="E25" s="223" t="inlineStr">
         <is>
-          <t>Net annual funding gap (base athletics)</t>
+          <t>comp @0</t>
         </is>
       </c>
-      <c r="C24" s="201">
-        <f>I18</f>
-        <v/>
-      </c>
-      <c r="K24" s="192" t="inlineStr">
+      <c r="F25" s="223" t="inlineStr">
         <is>
-          <t>This is the subsidy to run the full D1 program at conference-best BEFORE Making Cinderella content/sponsor revenue (SPV tabs) offsets it.</t>
+          <t>comp @50</t>
         </is>
       </c>
+      <c r="G25" s="223" t="inlineStr">
+        <is>
+          <t>comp @100</t>
+        </is>
+      </c>
+      <c r="H25" s="223" t="inlineStr">
+        <is>
+          <t>rev-share % of comp</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="224" t="inlineStr">
+        <is>
+          <t>Football</t>
+        </is>
+      </c>
+      <c r="C26" s="225">
+        <f>IF($C$9="FBS",C38,C37)</f>
+        <v/>
+      </c>
+      <c r="D26" s="225">
+        <f>IF($C$9="FBS",D38,D37)</f>
+        <v/>
+      </c>
+      <c r="E26" s="225">
+        <f>IF($C$9="FBS",E38,E37)</f>
+        <v/>
+      </c>
+      <c r="F26" s="225">
+        <f>IF($C$9="FBS",F38,F37)</f>
+        <v/>
+      </c>
+      <c r="G26" s="225">
+        <f>IF($C$9="FBS",G38,G37)</f>
+        <v/>
+      </c>
+      <c r="H26" s="226">
+        <f>IF($C$9="FBS",H38,H37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="224" t="inlineStr">
+        <is>
+          <t>Men's Basketball</t>
+        </is>
+      </c>
+      <c r="C27" s="227" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="D27" s="227" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="E27" s="227" t="n">
+        <v>400000</v>
+      </c>
+      <c r="F27" s="227" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="G27" s="227" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="H27" s="228" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="224" t="inlineStr">
+        <is>
+          <t>Women's Basketball</t>
+        </is>
+      </c>
+      <c r="C28" s="227" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="D28" s="227" t="n">
+        <v>400000</v>
+      </c>
+      <c r="E28" s="227" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F28" s="227" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="G28" s="227" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="H28" s="228" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L28" s="192" t="inlineStr">
+        <is>
+          <t>Subsidy to run the program at these dials BEFORE Making Cinderella content/sponsor revenue (SPV tabs) offsets it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="224" t="inlineStr">
+        <is>
+          <t>Baseball</t>
+        </is>
+      </c>
+      <c r="C29" s="227" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="D29" s="227" t="n">
+        <v>400000</v>
+      </c>
+      <c r="E29" s="227" t="n">
+        <v>250000</v>
+      </c>
+      <c r="F29" s="227" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="G29" s="227" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="H29" s="228" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="224" t="inlineStr">
+        <is>
+          <t>Softball</t>
+        </is>
+      </c>
+      <c r="C30" s="227" t="n">
+        <v>800000</v>
+      </c>
+      <c r="D30" s="227" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E30" s="227" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F30" s="227" t="n">
+        <v>600000</v>
+      </c>
+      <c r="G30" s="227" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="H30" s="228" t="n">
+        <v>0.667</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="224" t="inlineStr">
+        <is>
+          <t>Men's Soccer</t>
+        </is>
+      </c>
+      <c r="C31" s="227" t="n">
+        <v>700000</v>
+      </c>
+      <c r="D31" s="227" t="n">
+        <v>150000</v>
+      </c>
+      <c r="E31" s="227" t="n">
+        <v>120000</v>
+      </c>
+      <c r="F31" s="227" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G31" s="227" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="H31" s="228" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="224" t="inlineStr">
+        <is>
+          <t>Women's Soccer</t>
+        </is>
+      </c>
+      <c r="C32" s="227" t="n">
+        <v>700000</v>
+      </c>
+      <c r="D32" s="227" t="n">
+        <v>150000</v>
+      </c>
+      <c r="E32" s="227" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F32" s="227" t="n">
+        <v>400000</v>
+      </c>
+      <c r="G32" s="227" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="H32" s="228" t="n">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="224" t="inlineStr">
+        <is>
+          <t>Men's Lacrosse</t>
+        </is>
+      </c>
+      <c r="C33" s="227" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D33" s="227" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E33" s="227" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F33" s="227" t="n">
+        <v>600000</v>
+      </c>
+      <c r="G33" s="227" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="H33" s="228" t="n">
+        <v>0.583</v>
+      </c>
     </row>
     <row r="34">
-      <c r="B34" s="214" t="inlineStr">
+      <c r="B34" s="224" t="inlineStr">
         <is>
-          <t>FOOTBALL SCENARIO INPUTS (drive the Football row via the C5 toggle)</t>
+          <t>Women's Lacrosse</t>
         </is>
       </c>
-      <c r="C34" s="215" t="inlineStr"/>
-      <c r="D34" s="215" t="inlineStr"/>
-      <c r="E34" s="215" t="inlineStr"/>
-      <c r="F34" s="215" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="C35" s="216" t="inlineStr">
-        <is>
-          <t>Op cost</t>
-        </is>
-      </c>
-      <c r="D35" s="216" t="inlineStr">
-        <is>
-          <t>Team rev</t>
-        </is>
-      </c>
-      <c r="E35" s="216" t="inlineStr">
-        <is>
-          <t>Rev-share</t>
-        </is>
-      </c>
-      <c r="F35" s="216" t="inlineStr">
-        <is>
-          <t>NIL</t>
-        </is>
+      <c r="C34" s="227" t="n">
+        <v>800000</v>
+      </c>
+      <c r="D34" s="227" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E34" s="227" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F34" s="227" t="n">
+        <v>400000</v>
+      </c>
+      <c r="G34" s="227" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="H34" s="228" t="n">
+        <v>0.625</v>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="197" t="inlineStr">
         <is>
-          <t>FCS</t>
-        </is>
-      </c>
-      <c r="C36" s="196" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="D36" s="196" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="E36" s="196" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="F36" s="196" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="K36" s="192" t="inlineStr">
-        <is>
-          <t>FCS: 63 equiv. scholarships; 'guarantee games' vs FBS ($400-600K each) are real revenue.</t>
+          <t>Football scenario anchors (feed the Football engine row via the C9 toggle):</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="197" t="inlineStr">
         <is>
+          <t>FCS</t>
+        </is>
+      </c>
+      <c r="C37" s="196" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="D37" s="196" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="E37" s="196" t="n">
+        <v>750000</v>
+      </c>
+      <c r="F37" s="196" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="G37" s="196" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="H37" s="198" t="n">
+        <v>0.667</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="197" t="inlineStr">
+        <is>
           <t>FBS</t>
         </is>
       </c>
-      <c r="C37" s="196" t="n">
+      <c r="C38" s="196" t="n">
         <v>12000000</v>
       </c>
-      <c r="D37" s="196" t="n">
+      <c r="D38" s="196" t="n">
         <v>5000000</v>
       </c>
-      <c r="E37" s="196" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="F37" s="196" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="K37" s="192" t="inlineStr">
-        <is>
-          <t>FBS (Group-of-5-ish): comp near the whole House cap; a different qualification + capital path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="197" t="inlineStr">
-        <is>
-          <t>NOTES</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="186" t="inlineStr">
-        <is>
-          <t>• Columns 1-2 (op cost, team revenue) are the athletic PROGRAM view; columns 3-4 (rev-share, NIL) are athlete comp on top.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="186" t="inlineStr">
-        <is>
-          <t>• 'Competitive in conference' = clearly the best team in a low/mid-major (one-bid) league — NOT national-title spend.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="186" t="inlineStr">
-        <is>
-          <t>• Team revenue = base athletics only (tickets, guarantees, conference/unit distributions). Making Cinderella streaming/</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="186" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  sponsor/rev-share revenue is modeled in the SPV / SPV_D3 tabs and OFFSETS the net gap here — do not double-count.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="186" t="inlineStr">
-        <is>
-          <t>• Ramp over the reclassification arc: S1 (D3) ~12% of these figures; S2-S5 transition ramp; max in the first eligible</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="186" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  season (S6). This tab is the steady-state 'best-in-conference' snapshot; the year-by-year ramp is in the D3 memo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="186" t="inlineStr">
-        <is>
-          <t>• Figures are planning ranges from an opaque market (collectives don't disclose) — flex the blue inputs.</t>
-        </is>
+      <c r="E38" s="196" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="F38" s="196" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="G38" s="196" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="H38" s="198" t="n">
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C12 C13 C14 C15 C16 C17 C18 C19 C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="0-100 only" error="Effort must be 0-100." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add School_Ranking tab: 61-school weighted Cinderella-fit matrix
Five factors (Recruiting Draw, Win-Conversion, Sustainability, Monetization, Story Fit),
editable 1-10 scores + editable weights, live SCORE + RANK. Split 'winning' into
recruiting-draw x win-conversion per Norman; recalibrated Story to reward Americana/
regional-monopoly not just lost-glory; removed Patriot League (Holy Cross, Lehigh).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ajJRqKa1DUy4iKHJKPEi3
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-30-cinderella-model-d3-multisport.xlsx
+++ b/cinderella/Outputs/2026-07-30-cinderella-model-d3-multisport.xlsx
@@ -8,6 +8,7 @@
     <sheet name="SPV" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="SPV_D3" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="MultiSport" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="School_Ranking" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="RevSharePct">ASSUMPTIONS!$C$50</definedName>
@@ -649,7 +650,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="229">
+  <cellXfs count="235">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1233,6 +1234,24 @@
     <xf numFmtId="164" fontId="34" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="35" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="35" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="35" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="35" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="33" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -47940,4 +47959,2618 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:L73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" style="174" min="1" max="1"/>
+    <col width="20" customWidth="1" style="174" min="2" max="2"/>
+    <col width="12" customWidth="1" style="174" min="3" max="3"/>
+    <col width="11" customWidth="1" style="174" min="4" max="4"/>
+    <col width="11" customWidth="1" style="174" min="5" max="5"/>
+    <col width="11" customWidth="1" style="174" min="6" max="6"/>
+    <col width="11" customWidth="1" style="174" min="7" max="7"/>
+    <col width="11" customWidth="1" style="174" min="8" max="8"/>
+    <col width="9" customWidth="1" style="174" min="9" max="9"/>
+    <col width="7" customWidth="1" style="174" min="10" max="10"/>
+    <col width="44" customWidth="1" style="174" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="185" t="inlineStr">
+        <is>
+          <t>SCHOOL RANKING — CINDERELLA FIT (weighted scoring matrix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="186" t="inlineStr">
+        <is>
+          <t>Score each school 1-10 on the five factors (blue). Set the weights (yellow). Score + Rank recompute live. Re-order rows anytime via Data &gt; Sort by Score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="186" t="inlineStr">
+        <is>
+          <t>Celebrity NOT a factor (per Norman). $15M assumed for all — so 'winning' = Recruiting Draw (who'll choose you) x Win-Conversion (can the staff win with it), not raw money.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="197" t="inlineStr">
+        <is>
+          <t>FACTORS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="186" t="inlineStr">
+        <is>
+          <t>• Recruiting Draw: Would a top player CHOOSE here at equal money? Location, lifestyle, weather, campus, NBA-development appeal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="186" t="inlineStr">
+        <is>
+          <t>• Win-Conversion: Can the coach/program/culture turn talent into WINS? Coaching quality, hoops infrastructure, basketball DNA (football-first = lower).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="186" t="inlineStr">
+        <is>
+          <t>• Sustainability: Can it stay elite after Year 1? Institutional wealth/commitment, conference platform, donor+fan base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="186" t="inlineStr">
+        <is>
+          <t>• Monetization: Ability to MAKE money: media market, attendance/fanbase, conference $ + units, donor wealth, market monopoly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="186" t="inlineStr">
+        <is>
+          <t>• Story Fit: Cinderella storytelling: community texture, Americana / regional monopoly, lost-glory OR blank-slate. Never-won is neutral-to-positive, not a demerit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="197" t="inlineStr">
+        <is>
+          <t>WEIGHTS  (edit — need not sum to 100):</t>
+        </is>
+      </c>
+      <c r="D11" s="229" t="n">
+        <v>20</v>
+      </c>
+      <c r="E11" s="229" t="n">
+        <v>20</v>
+      </c>
+      <c r="F11" s="229" t="n">
+        <v>15</v>
+      </c>
+      <c r="G11" s="229" t="n">
+        <v>20</v>
+      </c>
+      <c r="H11" s="229" t="n">
+        <v>25</v>
+      </c>
+      <c r="I11" s="230">
+        <f>SUM(D11:H11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1" s="174">
+      <c r="B12" s="187" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="C12" s="231" t="inlineStr">
+        <is>
+          <t>Conf</t>
+        </is>
+      </c>
+      <c r="D12" s="210" t="inlineStr">
+        <is>
+          <t>Recruiting Draw</t>
+        </is>
+      </c>
+      <c r="E12" s="210" t="inlineStr">
+        <is>
+          <t>Win- Conversion</t>
+        </is>
+      </c>
+      <c r="F12" s="210" t="inlineStr">
+        <is>
+          <t>Sustain- ability</t>
+        </is>
+      </c>
+      <c r="G12" s="210" t="inlineStr">
+        <is>
+          <t>Monet- ization</t>
+        </is>
+      </c>
+      <c r="H12" s="210" t="inlineStr">
+        <is>
+          <t>Story Fit</t>
+        </is>
+      </c>
+      <c r="I12" s="210" t="inlineStr">
+        <is>
+          <t>SCORE</t>
+        </is>
+      </c>
+      <c r="J12" s="210" t="inlineStr">
+        <is>
+          <t>RANK</t>
+        </is>
+      </c>
+      <c r="L12" s="187" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="197" t="inlineStr">
+        <is>
+          <t>Tulane</t>
+        </is>
+      </c>
+      <c r="C13" s="232" t="inlineStr">
+        <is>
+          <t>AAC</t>
+        </is>
+      </c>
+      <c r="D13" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="I13" s="234">
+        <f>SUMPRODUCT(D13:H13,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J13" s="230">
+        <f>RANK(I13,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L13" s="192" t="inlineStr">
+        <is>
+          <t>New Orleans market/story/lifestyle; dormant giant</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="197" t="inlineStr">
+        <is>
+          <t>Loyola Marymount</t>
+        </is>
+      </c>
+      <c r="C14" s="232" t="inlineStr">
+        <is>
+          <t>WCC</t>
+        </is>
+      </c>
+      <c r="D14" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="G14" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I14" s="234">
+        <f>SUMPRODUCT(D14:H14,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J14" s="230">
+        <f>RANK(I14,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L14" s="192" t="inlineStr">
+        <is>
+          <t>LA market+lifestyle; '90 Gathers lore</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="197" t="inlineStr">
+        <is>
+          <t>Saint Joseph's</t>
+        </is>
+      </c>
+      <c r="C15" s="232" t="inlineStr">
+        <is>
+          <t>A-10</t>
+        </is>
+      </c>
+      <c r="D15" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F15" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="H15" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I15" s="234">
+        <f>SUMPRODUCT(D15:H15,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J15" s="230">
+        <f>RANK(I15,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L15" s="192" t="inlineStr">
+        <is>
+          <t>Philly + Big 5 tradition + A-10 units</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="197" t="inlineStr">
+        <is>
+          <t>Wichita State</t>
+        </is>
+      </c>
+      <c r="C16" s="232" t="inlineStr">
+        <is>
+          <t>AAC</t>
+        </is>
+      </c>
+      <c r="D16" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="F16" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I16" s="234">
+        <f>SUMPRODUCT(D16:H16,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J16" s="230">
+        <f>RANK(I16,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L16" s="192" t="inlineStr">
+        <is>
+          <t>Proven winner; rabid base+arena; heartland</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="197" t="inlineStr">
+        <is>
+          <t>Charleston</t>
+        </is>
+      </c>
+      <c r="C17" s="232" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="D17" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="E17" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F17" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="I17" s="234">
+        <f>SUMPRODUCT(D17:H17,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J17" s="230">
+        <f>RANK(I17,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L17" s="192" t="inlineStr">
+        <is>
+          <t>Charm/visuals/story; recent tourneys</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="197" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="C18" s="232" t="inlineStr">
+        <is>
+          <t>A-10</t>
+        </is>
+      </c>
+      <c r="D18" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="F18" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="G18" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="H18" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I18" s="234">
+        <f>SUMPRODUCT(D18:H18,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J18" s="230">
+        <f>RANK(I18,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L18" s="192" t="inlineStr">
+        <is>
+          <t>Elite wealth+academics; A-10; smart-underdog</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="197" t="inlineStr">
+        <is>
+          <t>Santa Clara</t>
+        </is>
+      </c>
+      <c r="C19" s="232" t="inlineStr">
+        <is>
+          <t>WCC</t>
+        </is>
+      </c>
+      <c r="D19" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="G19" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="H19" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I19" s="234">
+        <f>SUMPRODUCT(D19:H19,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J19" s="230">
+        <f>RANK(I19,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L19" s="192" t="inlineStr">
+        <is>
+          <t>Silicon Valley money/market; WCC hard to win</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="197" t="inlineStr">
+        <is>
+          <t>Providence</t>
+        </is>
+      </c>
+      <c r="C20" s="232" t="inlineStr">
+        <is>
+          <t>Big East</t>
+        </is>
+      </c>
+      <c r="D20" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="G20" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="H20" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I20" s="234">
+        <f>SUMPRODUCT(D20:H20,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J20" s="230">
+        <f>RANK(I20,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L20" s="192" t="inlineStr">
+        <is>
+          <t>Big East exposure/tradition; hard to win</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="197" t="inlineStr">
+        <is>
+          <t>Gonzaga</t>
+        </is>
+      </c>
+      <c r="C21" s="232" t="inlineStr">
+        <is>
+          <t>WCC</t>
+        </is>
+      </c>
+      <c r="D21" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="E21" s="233" t="n">
+        <v>10</v>
+      </c>
+      <c r="F21" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="G21" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="H21" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" s="234">
+        <f>SUMPRODUCT(D21:H21,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J21" s="230">
+        <f>RANK(I21,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L21" s="192" t="inlineStr">
+        <is>
+          <t>Elite program; ANTI-Cinderella (no transform)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="197" t="inlineStr">
+        <is>
+          <t>Belmont</t>
+        </is>
+      </c>
+      <c r="C22" s="232" t="inlineStr">
+        <is>
+          <t>MVC</t>
+        </is>
+      </c>
+      <c r="D22" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="F22" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="G22" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="H22" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I22" s="234">
+        <f>SUMPRODUCT(D22:H22,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J22" s="230">
+        <f>RANK(I22,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L22" s="192" t="inlineStr">
+        <is>
+          <t>Nashville market; strong program</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="197" t="inlineStr">
+        <is>
+          <t>Hawaii</t>
+        </is>
+      </c>
+      <c r="C23" s="232" t="inlineStr">
+        <is>
+          <t>Big West</t>
+        </is>
+      </c>
+      <c r="D23" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="E23" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H23" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="I23" s="234">
+        <f>SUMPRODUCT(D23:H23,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J23" s="230">
+        <f>RANK(I23,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L23" s="192" t="inlineStr">
+        <is>
+          <t>Islands lifestyle/story; market monopoly; travel caps $</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="197" t="inlineStr">
+        <is>
+          <t>Davidson</t>
+        </is>
+      </c>
+      <c r="C24" s="232" t="inlineStr">
+        <is>
+          <t>A-10</t>
+        </is>
+      </c>
+      <c r="D24" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="F24" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="G24" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H24" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I24" s="234">
+        <f>SUMPRODUCT(D24:H24,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J24" s="230">
+        <f>RANK(I24,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L24" s="192" t="inlineStr">
+        <is>
+          <t>Wealth/academics; already had its Cinderella</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="197" t="inlineStr">
+        <is>
+          <t>Pepperdine</t>
+        </is>
+      </c>
+      <c r="C25" s="232" t="inlineStr">
+        <is>
+          <t>WCC</t>
+        </is>
+      </c>
+      <c r="D25" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="E25" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="G25" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I25" s="234">
+        <f>SUMPRODUCT(D25:H25,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J25" s="230">
+        <f>RANK(I25,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L25" s="192" t="inlineStr">
+        <is>
+          <t>Malibu lifestyle/visuals; small base</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="197" t="inlineStr">
+        <is>
+          <t>Saint Louis</t>
+        </is>
+      </c>
+      <c r="C26" s="232" t="inlineStr">
+        <is>
+          <t>A-10</t>
+        </is>
+      </c>
+      <c r="D26" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E26" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="G26" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="H26" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I26" s="234">
+        <f>SUMPRODUCT(D26:H26,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J26" s="230">
+        <f>RANK(I26,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L26" s="192" t="inlineStr">
+        <is>
+          <t>St. Louis market; A-10; Catholic tradition</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="197" t="inlineStr">
+        <is>
+          <t>North Texas</t>
+        </is>
+      </c>
+      <c r="C27" s="232" t="inlineStr">
+        <is>
+          <t>AAC</t>
+        </is>
+      </c>
+      <c r="D27" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="E27" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="G27" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="H27" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I27" s="234">
+        <f>SUMPRODUCT(D27:H27,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J27" s="230">
+        <f>RANK(I27,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L27" s="192" t="inlineStr">
+        <is>
+          <t>DFW market; recent success; football-first</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="197" t="inlineStr">
+        <is>
+          <t>USC</t>
+        </is>
+      </c>
+      <c r="C28" s="232" t="inlineStr">
+        <is>
+          <t>Big Ten</t>
+        </is>
+      </c>
+      <c r="D28" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="E28" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="G28" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="H28" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="234">
+        <f>SUMPRODUCT(D28:H28,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J28" s="230">
+        <f>RANK(I28,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L28" s="192" t="inlineStr">
+        <is>
+          <t>LA giant; not an underdog</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="197" t="inlineStr">
+        <is>
+          <t>Saint Mary's</t>
+        </is>
+      </c>
+      <c r="C29" s="232" t="inlineStr">
+        <is>
+          <t>WCC</t>
+        </is>
+      </c>
+      <c r="D29" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="F29" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="G29" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H29" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I29" s="234">
+        <f>SUMPRODUCT(D29:H29,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J29" s="230">
+        <f>RANK(I29,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L29" s="192" t="inlineStr">
+        <is>
+          <t>Elite winner; weak story (arrived)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="197" t="inlineStr">
+        <is>
+          <t>Boston College</t>
+        </is>
+      </c>
+      <c r="C30" s="232" t="inlineStr">
+        <is>
+          <t>ACC</t>
+        </is>
+      </c>
+      <c r="D30" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="E30" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="G30" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="H30" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I30" s="234">
+        <f>SUMPRODUCT(D30:H30,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J30" s="230">
+        <f>RANK(I30,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L30" s="192" t="inlineStr">
+        <is>
+          <t>Boston + ACC money; fallen, not underdog</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="197" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="C31" s="232" t="inlineStr">
+        <is>
+          <t>WCC</t>
+        </is>
+      </c>
+      <c r="D31" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="E31" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="G31" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H31" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I31" s="234">
+        <f>SUMPRODUCT(D31:H31,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J31" s="230">
+        <f>RANK(I31,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L31" s="192" t="inlineStr">
+        <is>
+          <t>San Diego lifestyle/market; thin hoops tradition</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="197" t="inlineStr">
+        <is>
+          <t>Stanford</t>
+        </is>
+      </c>
+      <c r="C32" s="232" t="inlineStr">
+        <is>
+          <t>ACC</t>
+        </is>
+      </c>
+      <c r="D32" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="E32" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F32" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="G32" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="H32" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="I32" s="234">
+        <f>SUMPRODUCT(D32:H32,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J32" s="230">
+        <f>RANK(I32,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L32" s="192" t="inlineStr">
+        <is>
+          <t>Dormant giant; not an underdog</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="197" t="inlineStr">
+        <is>
+          <t>Fordham</t>
+        </is>
+      </c>
+      <c r="C33" s="232" t="inlineStr">
+        <is>
+          <t>A-10</t>
+        </is>
+      </c>
+      <c r="D33" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F33" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="G33" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="H33" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I33" s="234">
+        <f>SUMPRODUCT(D33:H33,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J33" s="230">
+        <f>RANK(I33,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L33" s="192" t="inlineStr">
+        <is>
+          <t>NYC market huge; program long dreadful (win risk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="197" t="inlineStr">
+        <is>
+          <t>Georgia State</t>
+        </is>
+      </c>
+      <c r="C34" s="232" t="inlineStr">
+        <is>
+          <t>Sun Belt</t>
+        </is>
+      </c>
+      <c r="D34" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="E34" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="H34" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I34" s="234">
+        <f>SUMPRODUCT(D34:H34,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J34" s="230">
+        <f>RANK(I34,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L34" s="192" t="inlineStr">
+        <is>
+          <t>Atlanta market; '15 lore; weak SB money</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="197" t="inlineStr">
+        <is>
+          <t>UC Irvine</t>
+        </is>
+      </c>
+      <c r="C35" s="232" t="inlineStr">
+        <is>
+          <t>Big West</t>
+        </is>
+      </c>
+      <c r="D35" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F35" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="G35" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H35" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I35" s="234">
+        <f>SUMPRODUCT(D35:H35,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J35" s="230">
+        <f>RANK(I35,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L35" s="192" t="inlineStr">
+        <is>
+          <t>Orange County lifestyle/market; solid</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="197" t="inlineStr">
+        <is>
+          <t>UMass</t>
+        </is>
+      </c>
+      <c r="C36" s="232" t="inlineStr">
+        <is>
+          <t>A-10</t>
+        </is>
+      </c>
+      <c r="D36" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F36" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="G36" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H36" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I36" s="234">
+        <f>SUMPRODUCT(D36:H36,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J36" s="230">
+        <f>RANK(I36,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L36" s="192" t="inlineStr">
+        <is>
+          <t>'96 Final Four fallen-giant; A-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="197" t="inlineStr">
+        <is>
+          <t>UTEP</t>
+        </is>
+      </c>
+      <c r="C37" s="232" t="inlineStr">
+        <is>
+          <t>C-USA</t>
+        </is>
+      </c>
+      <c r="D37" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G37" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H37" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="I37" s="234">
+        <f>SUMPRODUCT(D37:H37,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J37" s="230">
+        <f>RANK(I37,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L37" s="192" t="inlineStr">
+        <is>
+          <t>Glory Road '66 story + border-region monopoly</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="197" t="inlineStr">
+        <is>
+          <t>Texas Southern</t>
+        </is>
+      </c>
+      <c r="C38" s="232" t="inlineStr">
+        <is>
+          <t>SWAC</t>
+        </is>
+      </c>
+      <c r="D38" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E38" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G38" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H38" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="I38" s="234">
+        <f>SUMPRODUCT(D38:H38,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J38" s="230">
+        <f>RANK(I38,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L38" s="192" t="inlineStr">
+        <is>
+          <t>Houston + HBCU story; SWAC weak $</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="197" t="inlineStr">
+        <is>
+          <t>South Carolina</t>
+        </is>
+      </c>
+      <c r="C39" s="232" t="inlineStr">
+        <is>
+          <t>SEC</t>
+        </is>
+      </c>
+      <c r="D39" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E39" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F39" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="G39" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="H39" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I39" s="234">
+        <f>SUMPRODUCT(D39:H39,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J39" s="230">
+        <f>RANK(I39,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L39" s="192" t="inlineStr">
+        <is>
+          <t>SEC; football school; '17 Final Four</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="197" t="inlineStr">
+        <is>
+          <t>Wake Forest</t>
+        </is>
+      </c>
+      <c r="C40" s="232" t="inlineStr">
+        <is>
+          <t>ACC</t>
+        </is>
+      </c>
+      <c r="D40" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="G40" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H40" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I40" s="234">
+        <f>SUMPRODUCT(D40:H40,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J40" s="230">
+        <f>RANK(I40,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L40" s="192" t="inlineStr">
+        <is>
+          <t>ACC; Duncan lore; small market</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="197" t="inlineStr">
+        <is>
+          <t>Drake</t>
+        </is>
+      </c>
+      <c r="C41" s="232" t="inlineStr">
+        <is>
+          <t>MVC</t>
+        </is>
+      </c>
+      <c r="D41" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E41" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F41" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="G41" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H41" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I41" s="234">
+        <f>SUMPRODUCT(D41:H41,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J41" s="230">
+        <f>RANK(I41,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L41" s="192" t="inlineStr">
+        <is>
+          <t>MVC winner; Des Moines heartland</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="197" t="inlineStr">
+        <is>
+          <t>Tennessee State</t>
+        </is>
+      </c>
+      <c r="C42" s="232" t="inlineStr">
+        <is>
+          <t>Big South</t>
+        </is>
+      </c>
+      <c r="D42" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E42" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H42" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="I42" s="234">
+        <f>SUMPRODUCT(D42:H42,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J42" s="230">
+        <f>RANK(I42,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L42" s="192" t="inlineStr">
+        <is>
+          <t>Nashville + HBCU story; low conf $</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="197" t="inlineStr">
+        <is>
+          <t>Northeastern</t>
+        </is>
+      </c>
+      <c r="C43" s="232" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="D43" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="E43" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="G43" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H43" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I43" s="234">
+        <f>SUMPRODUCT(D43:H43,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J43" s="230">
+        <f>RANK(I43,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L43" s="192" t="inlineStr">
+        <is>
+          <t>Boston market; academics</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="197" t="inlineStr">
+        <is>
+          <t>Rhode Island</t>
+        </is>
+      </c>
+      <c r="C44" s="232" t="inlineStr">
+        <is>
+          <t>A-10</t>
+        </is>
+      </c>
+      <c r="D44" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E44" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F44" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="G44" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H44" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I44" s="234">
+        <f>SUMPRODUCT(D44:H44,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J44" s="230">
+        <f>RANK(I44,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L44" s="192" t="inlineStr">
+        <is>
+          <t>A-10; recent Hurley-era success</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="197" t="inlineStr">
+        <is>
+          <t>Indiana State</t>
+        </is>
+      </c>
+      <c r="C45" s="232" t="inlineStr">
+        <is>
+          <t>MVC</t>
+        </is>
+      </c>
+      <c r="D45" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E45" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F45" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G45" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H45" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I45" s="234">
+        <f>SUMPRODUCT(D45:H45,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J45" s="230">
+        <f>RANK(I45,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L45" s="192" t="inlineStr">
+        <is>
+          <t>Heartland lore; '24 near-miss</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="197" t="inlineStr">
+        <is>
+          <t>Furman</t>
+        </is>
+      </c>
+      <c r="C46" s="232" t="inlineStr">
+        <is>
+          <t>SoCon</t>
+        </is>
+      </c>
+      <c r="D46" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E46" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F46" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G46" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H46" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I46" s="234">
+        <f>SUMPRODUCT(D46:H46,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J46" s="230">
+        <f>RANK(I46,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L46" s="192" t="inlineStr">
+        <is>
+          <t>Charm; '23 upset; Greenville</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="197" t="inlineStr">
+        <is>
+          <t>William &amp; Mary</t>
+        </is>
+      </c>
+      <c r="C47" s="232" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="D47" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F47" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="G47" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H47" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I47" s="234">
+        <f>SUMPRODUCT(D47:H47,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J47" s="230">
+        <f>RANK(I47,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L47" s="192" t="inlineStr">
+        <is>
+          <t>Historic charm; small market</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="197" t="inlineStr">
+        <is>
+          <t>High Point</t>
+        </is>
+      </c>
+      <c r="C48" s="232" t="inlineStr">
+        <is>
+          <t>Big South</t>
+        </is>
+      </c>
+      <c r="D48" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F48" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="G48" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H48" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I48" s="234">
+        <f>SUMPRODUCT(D48:H48,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J48" s="230">
+        <f>RANK(I48,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L48" s="192" t="inlineStr">
+        <is>
+          <t>Already investing; new arena; small market</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="197" t="inlineStr">
+        <is>
+          <t>McNeese State</t>
+        </is>
+      </c>
+      <c r="C49" s="232" t="inlineStr">
+        <is>
+          <t>Southland</t>
+        </is>
+      </c>
+      <c r="D49" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F49" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G49" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H49" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I49" s="234">
+        <f>SUMPRODUCT(D49:H49,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J49" s="230">
+        <f>RANK(I49,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L49" s="192" t="inlineStr">
+        <is>
+          <t>Recent Cinderella; Louisiana Americana; tiny $</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="197" t="inlineStr">
+        <is>
+          <t>New Hampshire</t>
+        </is>
+      </c>
+      <c r="C50" s="232" t="inlineStr">
+        <is>
+          <t>America East</t>
+        </is>
+      </c>
+      <c r="D50" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F50" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G50" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H50" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="I50" s="234">
+        <f>SUMPRODUCT(D50:H50,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J50" s="230">
+        <f>RANK(I50,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L50" s="192" t="inlineStr">
+        <is>
+          <t>Forgotten-Americana + state sports monopoly</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="197" t="inlineStr">
+        <is>
+          <t>Detroit</t>
+        </is>
+      </c>
+      <c r="C51" s="232" t="inlineStr">
+        <is>
+          <t>Horizon</t>
+        </is>
+      </c>
+      <c r="D51" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E51" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G51" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H51" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I51" s="234">
+        <f>SUMPRODUCT(D51:H51,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J51" s="230">
+        <f>RANK(I51,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L51" s="192" t="inlineStr">
+        <is>
+          <t>Detroit market; dormant; urban story</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="197" t="inlineStr">
+        <is>
+          <t>New Orleans</t>
+        </is>
+      </c>
+      <c r="C52" s="232" t="inlineStr">
+        <is>
+          <t>Southland</t>
+        </is>
+      </c>
+      <c r="D52" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="E52" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H52" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I52" s="234">
+        <f>SUMPRODUCT(D52:H52,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J52" s="230">
+        <f>RANK(I52,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L52" s="192" t="inlineStr">
+        <is>
+          <t>NOLA market/story; weak program (Tulane better)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="197" t="inlineStr">
+        <is>
+          <t>Hofstra</t>
+        </is>
+      </c>
+      <c r="C53" s="232" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="D53" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E53" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F53" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G53" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H53" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I53" s="234">
+        <f>SUMPRODUCT(D53:H53,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J53" s="230">
+        <f>RANK(I53,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L53" s="192" t="inlineStr">
+        <is>
+          <t>NYC-area market; CAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="197" t="inlineStr">
+        <is>
+          <t>ETSU</t>
+        </is>
+      </c>
+      <c r="C54" s="232" t="inlineStr">
+        <is>
+          <t>SoCon</t>
+        </is>
+      </c>
+      <c r="D54" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E54" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F54" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H54" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="I54" s="234">
+        <f>SUMPRODUCT(D54:H54,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J54" s="230">
+        <f>RANK(I54,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L54" s="192" t="inlineStr">
+        <is>
+          <t>Appalachia Americana; hoops history</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="197" t="inlineStr">
+        <is>
+          <t>Oregon State</t>
+        </is>
+      </c>
+      <c r="C55" s="232" t="inlineStr">
+        <is>
+          <t>WCC</t>
+        </is>
+      </c>
+      <c r="D55" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E55" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F55" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="G55" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H55" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I55" s="234">
+        <f>SUMPRODUCT(D55:H55,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J55" s="230">
+        <f>RANK(I55,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L55" s="192" t="inlineStr">
+        <is>
+          <t>Pac-12 orphan; Payton lore; messy</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="197" t="inlineStr">
+        <is>
+          <t>UNC Greensboro</t>
+        </is>
+      </c>
+      <c r="C56" s="232" t="inlineStr">
+        <is>
+          <t>SoCon</t>
+        </is>
+      </c>
+      <c r="D56" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E56" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F56" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G56" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H56" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I56" s="234">
+        <f>SUMPRODUCT(D56:H56,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J56" s="230">
+        <f>RANK(I56,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L56" s="192" t="inlineStr">
+        <is>
+          <t>Solid SoCon; modest ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="197" t="inlineStr">
+        <is>
+          <t>Texas State</t>
+        </is>
+      </c>
+      <c r="C57" s="232" t="inlineStr">
+        <is>
+          <t>Sun Belt</t>
+        </is>
+      </c>
+      <c r="D57" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E57" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F57" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G57" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="H57" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I57" s="234">
+        <f>SUMPRODUCT(D57:H57,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J57" s="230">
+        <f>RANK(I57,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L57" s="192" t="inlineStr">
+        <is>
+          <t>Austin-area growth; football-first</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="197" t="inlineStr">
+        <is>
+          <t>Weber State</t>
+        </is>
+      </c>
+      <c r="C58" s="232" t="inlineStr">
+        <is>
+          <t>Big Sky</t>
+        </is>
+      </c>
+      <c r="D58" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E58" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F58" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G58" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H58" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I58" s="234">
+        <f>SUMPRODUCT(D58:H58,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J58" s="230">
+        <f>RANK(I58,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L58" s="192" t="inlineStr">
+        <is>
+          <t>Guard lore; Ogden; mountain Americana</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="197" t="inlineStr">
+        <is>
+          <t>Appalachian State</t>
+        </is>
+      </c>
+      <c r="C59" s="232" t="inlineStr">
+        <is>
+          <t>Sun Belt</t>
+        </is>
+      </c>
+      <c r="D59" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E59" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F59" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G59" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H59" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="I59" s="234">
+        <f>SUMPRODUCT(D59:H59,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J59" s="230">
+        <f>RANK(I59,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L59" s="192" t="inlineStr">
+        <is>
+          <t>Boone mountain Americana; thin hoops</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="197" t="inlineStr">
+        <is>
+          <t>Denver</t>
+        </is>
+      </c>
+      <c r="C60" s="232" t="inlineStr">
+        <is>
+          <t>Summit</t>
+        </is>
+      </c>
+      <c r="D60" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="E60" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F60" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G60" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H60" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I60" s="234">
+        <f>SUMPRODUCT(D60:H60,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J60" s="230">
+        <f>RANK(I60,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L60" s="192" t="inlineStr">
+        <is>
+          <t>Good market/lifestyle; ~zero hoops base</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="197" t="inlineStr">
+        <is>
+          <t>Missouri State</t>
+        </is>
+      </c>
+      <c r="C61" s="232" t="inlineStr">
+        <is>
+          <t>C-USA</t>
+        </is>
+      </c>
+      <c r="D61" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E61" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F61" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G61" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H61" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I61" s="234">
+        <f>SUMPRODUCT(D61:H61,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J61" s="230">
+        <f>RANK(I61,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L61" s="192" t="inlineStr">
+        <is>
+          <t>Solid mid-major; medium market</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="197" t="inlineStr">
+        <is>
+          <t>Fairfield</t>
+        </is>
+      </c>
+      <c r="C62" s="232" t="inlineStr">
+        <is>
+          <t>MAAC</t>
+        </is>
+      </c>
+      <c r="D62" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E62" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F62" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G62" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H62" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I62" s="234">
+        <f>SUMPRODUCT(D62:H62,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J62" s="230">
+        <f>RANK(I62,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L62" s="192" t="inlineStr">
+        <is>
+          <t>Wealthy CT; MAAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="197" t="inlineStr">
+        <is>
+          <t>Kent State</t>
+        </is>
+      </c>
+      <c r="C63" s="232" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="D63" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E63" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F63" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G63" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H63" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I63" s="234">
+        <f>SUMPRODUCT(D63:H63,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J63" s="230">
+        <f>RANK(I63,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L63" s="192" t="inlineStr">
+        <is>
+          <t>MAC; '02 Elite Eight lore</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="197" t="inlineStr">
+        <is>
+          <t>LIU</t>
+        </is>
+      </c>
+      <c r="C64" s="232" t="inlineStr">
+        <is>
+          <t>NEC</t>
+        </is>
+      </c>
+      <c r="D64" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="E64" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="F64" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="G64" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H64" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I64" s="234">
+        <f>SUMPRODUCT(D64:H64,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J64" s="230">
+        <f>RANK(I64,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L64" s="192" t="inlineStr">
+        <is>
+          <t>Brooklyn market; NEC/no infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="197" t="inlineStr">
+        <is>
+          <t>UMKC</t>
+        </is>
+      </c>
+      <c r="C65" s="232" t="inlineStr">
+        <is>
+          <t>Summit</t>
+        </is>
+      </c>
+      <c r="D65" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E65" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G65" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H65" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I65" s="234">
+        <f>SUMPRODUCT(D65:H65,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J65" s="230">
+        <f>RANK(I65,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L65" s="192" t="inlineStr">
+        <is>
+          <t>KC market; weak program</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="197" t="inlineStr">
+        <is>
+          <t>Georgia Southern</t>
+        </is>
+      </c>
+      <c r="C66" s="232" t="inlineStr">
+        <is>
+          <t>Sun Belt</t>
+        </is>
+      </c>
+      <c r="D66" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E66" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F66" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G66" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="H66" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I66" s="234">
+        <f>SUMPRODUCT(D66:H66,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J66" s="230">
+        <f>RANK(I66,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L66" s="192" t="inlineStr">
+        <is>
+          <t>Football-first</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="197" t="inlineStr">
+        <is>
+          <t>Elon</t>
+        </is>
+      </c>
+      <c r="C67" s="232" t="inlineStr">
+        <is>
+          <t>CAA</t>
+        </is>
+      </c>
+      <c r="D67" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="E67" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F67" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="G67" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H67" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I67" s="234">
+        <f>SUMPRODUCT(D67:H67,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J67" s="230">
+        <f>RANK(I67,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L67" s="192" t="inlineStr">
+        <is>
+          <t>Nice academics; no hoops relevance</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="197" t="inlineStr">
+        <is>
+          <t>Miami (OH)</t>
+        </is>
+      </c>
+      <c r="C68" s="232" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="D68" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E68" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F68" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G68" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="H68" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="I68" s="234">
+        <f>SUMPRODUCT(D68:H68,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J68" s="230">
+        <f>RANK(I68,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L68" s="192" t="inlineStr">
+        <is>
+          <t>Cradle of coaches; tiny market</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="197" t="inlineStr">
+        <is>
+          <t>Ball State</t>
+        </is>
+      </c>
+      <c r="C69" s="232" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="D69" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E69" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F69" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G69" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H69" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I69" s="234">
+        <f>SUMPRODUCT(D69:H69,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J69" s="230">
+        <f>RANK(I69,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L69" s="192" t="inlineStr">
+        <is>
+          <t>MAC; small market</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="197" t="inlineStr">
+        <is>
+          <t>Marist</t>
+        </is>
+      </c>
+      <c r="C70" s="232" t="inlineStr">
+        <is>
+          <t>MAAC</t>
+        </is>
+      </c>
+      <c r="D70" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E70" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F70" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G70" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H70" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I70" s="234">
+        <f>SUMPRODUCT(D70:H70,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J70" s="230">
+        <f>RANK(I70,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L70" s="192" t="inlineStr">
+        <is>
+          <t>Small MAAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="197" t="inlineStr">
+        <is>
+          <t>Northern Illinois</t>
+        </is>
+      </c>
+      <c r="C71" s="232" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="D71" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="E71" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F71" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="G71" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="H71" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="I71" s="234">
+        <f>SUMPRODUCT(D71:H71,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J71" s="230">
+        <f>RANK(I71,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L71" s="192" t="inlineStr">
+        <is>
+          <t>Weak hoops</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="197" t="inlineStr">
+        <is>
+          <t>Central Arkansas</t>
+        </is>
+      </c>
+      <c r="C72" s="232" t="inlineStr">
+        <is>
+          <t>ASUN</t>
+        </is>
+      </c>
+      <c r="D72" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="E72" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F72" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="G72" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="H72" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I72" s="234">
+        <f>SUMPRODUCT(D72:H72,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J72" s="230">
+        <f>RANK(I72,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L72" s="192" t="inlineStr">
+        <is>
+          <t>Weak conference/market</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="197" t="inlineStr">
+        <is>
+          <t>Louisiana Monroe</t>
+        </is>
+      </c>
+      <c r="C73" s="232" t="inlineStr">
+        <is>
+          <t>Sun Belt</t>
+        </is>
+      </c>
+      <c r="D73" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="E73" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="F73" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="G73" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="H73" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="I73" s="234">
+        <f>SUMPRODUCT(D73:H73,$D$11:$H$11)/SUM($D$11:$H$11)</f>
+        <v/>
+      </c>
+      <c r="J73" s="230">
+        <f>RANK(I73,$I$13:$I$73)</f>
+        <v/>
+      </c>
+      <c r="L73" s="192" t="inlineStr">
+        <is>
+          <t>Weak everything</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 F41 F42 F43 F44 F45 F46 F47 F48 F49 F50 F51 F52 F53 F54 F55 F56 F57 F58 F59 F60 F61 F62 F63 F64 F65 F66 F67 F68 F69 F70 F71 F72 F73 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45 G46 G47 G48 G49 G50 G51 G52 G53 G54 G55 G56 G57 G58 G59 G60 G61 G62 G63 G64 G65 G66 G67 G68 G69 G70 G71 G72 G73 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="1-10" error="Score 1-10 only" type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>